<commit_message>
feat : inventory ui
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/EquipItemInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/EquipItemInfo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514B0CFA-D19B-42FD-8079-36171657026D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EAFC925-1894-4F51-A83C-7E305DF46EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{3510F260-6A7D-4843-A2DA-E1BA315C89A0}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="42">
   <si>
     <t>int</t>
   </si>
@@ -45,18 +45,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>List&lt;int&gt;</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>OptionCount</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>OptionPoolID</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>Level</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -73,30 +61,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>MinValue</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>MaxValue</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>효과 최소 값</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>효과 최대값</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>옵션 개수</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>옵션 풀</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>착용제한 레벨</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -117,14 +81,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>스텟 옵션키</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>StatEffectID</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>Enum&lt;EquipType&gt;</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -177,15 +133,59 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>List&lt;Enum&lt;StatType&gt;&gt;</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>PhysicalDefence</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>PhysicalAttack</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxHp</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxMp</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxShield</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxHunger</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MagicalAttack</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MagicalDefence</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>CriticalChance</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>CriticalMultiplier</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>float</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>백분율</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>고정상수</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1161,67 +1161,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27433482-0B68-4763-85C6-CA814D549BDC}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="9" style="1"/>
-    <col min="8" max="8" width="9.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="1" max="4" width="9" style="1"/>
+    <col min="6" max="8" width="9" style="1"/>
+    <col min="9" max="9" width="9.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>34</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>2</v>
@@ -1232,389 +1248,584 @@
       <c r="J2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="K2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>19</v>
+        <v>40</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>101</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>2</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>201</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
-        <v>2</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>301</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
-        <v>2</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>401</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
-        <v>2</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>501</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <v>2</v>
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>601</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>2</v>
+        <v>21</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>701</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="1">
+        <v>22</v>
+      </c>
+      <c r="E10">
         <v>0</v>
       </c>
-      <c r="G10" s="1">
-        <v>2</v>
+      <c r="F10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>801</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F11" s="1">
+        <v>23</v>
+      </c>
+      <c r="E11">
         <v>0</v>
       </c>
-      <c r="G11" s="1">
-        <v>2</v>
+      <c r="F11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>901</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="1">
+        <v>24</v>
+      </c>
+      <c r="E12">
         <v>0</v>
       </c>
-      <c r="G12" s="1">
-        <v>2</v>
+      <c r="F12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1001</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="1">
+        <v>25</v>
+      </c>
+      <c r="E13">
         <v>0</v>
       </c>
-      <c r="G13" s="1">
-        <v>2</v>
+      <c r="F13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1101</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="1">
+        <v>26</v>
+      </c>
+      <c r="E14">
         <v>0</v>
       </c>
-      <c r="G14" s="1">
-        <v>2</v>
+      <c r="F14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>